<commit_message>
panchapale given menaka dd continue
</commit_message>
<xml_diff>
--- a/drg/menaka dd/archi/calculations load/wall load calculation.xlsx
+++ b/drg/menaka dd/archi/calculations load/wall load calculation.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933A39FF-BCB5-43D5-99B6-DCBA8E45228F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A79D762C-B6B5-4FCB-89B1-23B397B93E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="5985" yWindow="1095" windowWidth="13050" windowHeight="10050" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Interpoaltion" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="61">
   <si>
     <t>y-y1=((y2-y1)/(x2-x1))*(x-x1)</t>
   </si>
@@ -933,7 +933,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CF5F103-52A0-4D11-811D-43BFE2FAABA8}">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -946,9 +946,16 @@
     <col min="9" max="9" width="11" customWidth="1"/>
     <col min="10" max="11" width="11" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8" customWidth="1"/>
+    <col min="17" max="17" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="30" t="s">
         <v>3</v>
       </c>
@@ -972,8 +979,31 @@
       <c r="I1" s="32"/>
       <c r="J1" s="32"/>
       <c r="K1" s="32"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M1" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="N1" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q1" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" s="31"/>
+      <c r="S1" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
+    </row>
+    <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="30"/>
       <c r="B2" s="30"/>
       <c r="C2" s="3" t="s">
@@ -997,8 +1027,31 @@
         <v>30</v>
       </c>
       <c r="K2" s="34"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="S2" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="T2" s="34"/>
+      <c r="U2" s="15"/>
+      <c r="V2" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="W2" s="34"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="3"/>
@@ -1018,8 +1071,27 @@
       <c r="K3" s="11" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="U3" s="16"/>
+      <c r="V3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="W3" s="11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
@@ -1057,8 +1129,45 @@
         <f>0.75*H4</f>
         <v>9.0258900000000022</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="M4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" s="2">
+        <v>20</v>
+      </c>
+      <c r="P4" s="2">
+        <v>0.23</v>
+      </c>
+      <c r="Q4" s="2">
+        <f>Q15</f>
+        <v>2.3113999999999999</v>
+      </c>
+      <c r="R4" s="14">
+        <f>Q16</f>
+        <v>2.6162000000000001</v>
+      </c>
+      <c r="S4" s="12">
+        <f>P4*Q4*O4</f>
+        <v>10.632440000000001</v>
+      </c>
+      <c r="T4" s="13">
+        <f>P4*R4*O4</f>
+        <v>12.034520000000002</v>
+      </c>
+      <c r="U4" s="17"/>
+      <c r="V4" s="12">
+        <f>0.75*S4</f>
+        <v>7.9743300000000001</v>
+      </c>
+      <c r="W4" s="13">
+        <f>0.75*T4</f>
+        <v>9.0258900000000022</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
@@ -1092,8 +1201,41 @@
         <f>0.75*H5</f>
         <v>9.0258900000000022</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2">
+        <f>Q17</f>
+        <v>2.3113999999999999</v>
+      </c>
+      <c r="R5" s="14">
+        <f>Q18</f>
+        <v>2.6162000000000001</v>
+      </c>
+      <c r="S5" s="12">
+        <f>P4*Q5*O4</f>
+        <v>10.632440000000001</v>
+      </c>
+      <c r="T5" s="13">
+        <f>P4*R5*O4</f>
+        <v>12.034520000000002</v>
+      </c>
+      <c r="U5" s="17"/>
+      <c r="V5" s="12">
+        <f>0.75*S5</f>
+        <v>7.9743300000000001</v>
+      </c>
+      <c r="W5" s="13">
+        <f>0.75*T5</f>
+        <v>9.0258900000000022</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="1"/>
       <c r="C6" s="2"/>
@@ -1105,8 +1247,19 @@
       <c r="I6" s="17"/>
       <c r="J6" s="12"/>
       <c r="K6" s="13"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M6" s="3"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="13"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="12"/>
+      <c r="W6" s="13"/>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
@@ -1144,8 +1297,45 @@
         <f>0.75*H7</f>
         <v>4.5129450000000011</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="M7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" s="2">
+        <v>20</v>
+      </c>
+      <c r="P7" s="2">
+        <v>0.115</v>
+      </c>
+      <c r="Q7" s="2">
+        <f>Q4</f>
+        <v>2.3113999999999999</v>
+      </c>
+      <c r="R7" s="14">
+        <f>R4</f>
+        <v>2.6162000000000001</v>
+      </c>
+      <c r="S7" s="12">
+        <f>P7*Q7*O7</f>
+        <v>5.3162200000000004</v>
+      </c>
+      <c r="T7" s="13">
+        <f>P7*R7*O7</f>
+        <v>6.0172600000000012</v>
+      </c>
+      <c r="U7" s="17"/>
+      <c r="V7" s="12">
+        <f>0.75*S7</f>
+        <v>3.9871650000000001</v>
+      </c>
+      <c r="W7" s="13">
+        <f>0.75*T7</f>
+        <v>4.5129450000000011</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
@@ -1179,8 +1369,41 @@
         <f>0.75*H8</f>
         <v>4.5129450000000011</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2">
+        <f>Q5</f>
+        <v>2.3113999999999999</v>
+      </c>
+      <c r="R8" s="14">
+        <f>R5</f>
+        <v>2.6162000000000001</v>
+      </c>
+      <c r="S8" s="12">
+        <f>P7*Q8*O7</f>
+        <v>5.3162200000000004</v>
+      </c>
+      <c r="T8" s="13">
+        <f>P7*R8*O7</f>
+        <v>6.0172600000000012</v>
+      </c>
+      <c r="U8" s="17"/>
+      <c r="V8" s="12">
+        <f>0.75*S8</f>
+        <v>3.9871650000000001</v>
+      </c>
+      <c r="W8" s="13">
+        <f>0.75*T8</f>
+        <v>4.5129450000000011</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="1"/>
       <c r="C9" s="2"/>
@@ -1192,8 +1415,19 @@
       <c r="I9" s="20"/>
       <c r="J9" s="18"/>
       <c r="K9" s="19"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M9" s="3"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="14"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="20"/>
+      <c r="V9" s="18"/>
+      <c r="W9" s="19"/>
+    </row>
+    <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
@@ -1219,8 +1453,33 @@
       <c r="I10" s="36"/>
       <c r="J10" s="36"/>
       <c r="K10" s="37"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O10" s="2">
+        <v>20</v>
+      </c>
+      <c r="P10" s="2">
+        <v>0.115</v>
+      </c>
+      <c r="Q10" s="28">
+        <f>Q19</f>
+        <v>0.91439999999999999</v>
+      </c>
+      <c r="R10" s="29"/>
+      <c r="S10" s="35">
+        <f>P10*Q10*O10</f>
+        <v>2.1031200000000001</v>
+      </c>
+      <c r="T10" s="36"/>
+      <c r="U10" s="36"/>
+      <c r="V10" s="36"/>
+      <c r="W10" s="37"/>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
@@ -1231,8 +1490,18 @@
       <c r="E14" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="N14" s="8"/>
+      <c r="P14" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1244,8 +1513,19 @@
         <f>CONVERT(D15,"in","m")</f>
         <v>2.3875999999999999</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P15" s="1">
+        <f>7*12+7</f>
+        <v>91</v>
+      </c>
+      <c r="Q15" s="2">
+        <f>CONVERT(P15,"in","m")</f>
+        <v>2.3113999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="D16" s="1">
         <f>8*12+7</f>
         <v>103</v>
@@ -1254,8 +1534,16 @@
         <f>CONVERT(D16,"in","m")</f>
         <v>2.6162000000000001</v>
       </c>
-    </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="P16" s="1">
+        <f>8*12+7</f>
+        <v>103</v>
+      </c>
+      <c r="Q16" s="2">
+        <f>CONVERT(P16,"in","m")</f>
+        <v>2.6162000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D17" s="1">
         <f>7*12+10</f>
         <v>94</v>
@@ -1264,8 +1552,16 @@
         <f>CONVERT(D17,"in","m")</f>
         <v>2.3875999999999999</v>
       </c>
-    </row>
-    <row r="18" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="P17" s="1">
+        <f>7*12+7</f>
+        <v>91</v>
+      </c>
+      <c r="Q17" s="2">
+        <f>CONVERT(P17,"in","m")</f>
+        <v>2.3113999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D18" s="1">
         <f>8*12+7</f>
         <v>103</v>
@@ -1274,8 +1570,16 @@
         <f>CONVERT(D18,"in","m")</f>
         <v>2.6162000000000001</v>
       </c>
-    </row>
-    <row r="19" spans="4:5" x14ac:dyDescent="0.25">
+      <c r="P18" s="1">
+        <f>8*12+7</f>
+        <v>103</v>
+      </c>
+      <c r="Q18" s="2">
+        <f>CONVERT(P18,"in","m")</f>
+        <v>2.6162000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="4:17" x14ac:dyDescent="0.25">
       <c r="D19" s="1">
         <f>3*12</f>
         <v>36</v>
@@ -1284,9 +1588,25 @@
         <f>CONVERT(D19,"in","m")</f>
         <v>0.91439999999999999</v>
       </c>
+      <c r="P19" s="1">
+        <f>3*12</f>
+        <v>36</v>
+      </c>
+      <c r="Q19" s="2">
+        <f>CONVERT(P19,"in","m")</f>
+        <v>0.91439999999999999</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="16">
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="M1:M2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="S1:W1"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="V2:W2"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="E1:F1"/>

</xml_diff>